<commit_message>
Atualiza dados do estoque e compras3
</commit_message>
<xml_diff>
--- a/data-source/ESTOQUEPARAGUAI.xlsx
+++ b/data-source/ESTOQUEPARAGUAI.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/Relatórios SMART-STOCK/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/SMART-STOCK/data-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{EB3E627F-C983-4B18-AD05-2EA6762DAB6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6AEBD3E-12D8-4064-AC76-3FB9834E7C81}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{EB3E627F-C983-4B18-AD05-2EA6762DAB6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73EBB94A-344A-4CF6-BAFF-811B61FB52E8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A9832E4A-FA62-42FB-B6CE-C34852AF63FE}"/>
   </bookViews>
@@ -20,6 +20,17 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
     </ext>
@@ -28,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="15">
   <si>
     <t>Grupo</t>
   </si>
@@ -120,16 +131,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -492,309 +501,323 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="4">
+      <c r="A2" s="2">
         <v>9073</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="6">
+      <c r="B2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2">
         <v>780</v>
       </c>
-      <c r="D2" s="6">
-        <v>13</v>
-      </c>
-      <c r="E2" s="6" t="s">
+      <c r="D2">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="4">
+      <c r="A3" s="2">
         <v>6520</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3">
         <v>16154</v>
       </c>
-      <c r="D3" s="6">
-        <v>13</v>
-      </c>
-      <c r="E3" s="6" t="s">
+      <c r="D3">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="4">
+      <c r="A4" s="2">
         <v>6518</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4">
         <v>2842</v>
       </c>
-      <c r="D4" s="6">
-        <v>13</v>
-      </c>
-      <c r="E4" s="6" t="s">
+      <c r="D4">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="4">
+      <c r="A5" s="2">
         <v>9073</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="6">
+      <c r="B5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5">
         <v>24584</v>
       </c>
-      <c r="D5" s="6">
-        <v>13</v>
-      </c>
-      <c r="E5" s="6" t="s">
+      <c r="D5">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="4">
+      <c r="A6" s="2">
         <v>9073</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="6">
+      <c r="B6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6">
         <v>3960</v>
       </c>
-      <c r="D6" s="6">
-        <v>13</v>
-      </c>
-      <c r="E6" s="6" t="s">
+      <c r="D6">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="4">
+      <c r="A7" s="2">
         <v>9073</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="6">
+      <c r="B7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7">
         <v>16000</v>
       </c>
-      <c r="D7" s="6">
-        <v>13</v>
-      </c>
-      <c r="E7" s="6" t="s">
+      <c r="D7">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="4">
+      <c r="A8" s="2">
         <v>15721</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8">
         <v>8200</v>
       </c>
-      <c r="D8" s="6">
-        <v>13</v>
-      </c>
-      <c r="E8" s="6" t="s">
+      <c r="D8">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
+      <c r="A9" s="2">
         <v>9010</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9">
         <v>3243</v>
       </c>
-      <c r="D9" s="6">
-        <v>13</v>
-      </c>
-      <c r="E9" s="6" t="s">
+      <c r="D9">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="4">
+      <c r="A10" s="2">
         <v>9073</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="6">
+      <c r="B10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10">
         <v>30795</v>
       </c>
-      <c r="D10" s="6">
-        <v>13</v>
-      </c>
-      <c r="E10" s="6" t="s">
+      <c r="D10">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="4">
+      <c r="A11" s="2">
         <v>10608</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11">
         <v>11279</v>
       </c>
-      <c r="D11" s="6">
-        <v>13</v>
-      </c>
-      <c r="E11" s="6" t="s">
+      <c r="D11">
+        <v>13</v>
+      </c>
+      <c r="E11" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="4">
+      <c r="A12" s="2">
         <v>9004</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12">
         <v>10303</v>
       </c>
-      <c r="D12" s="6">
-        <v>13</v>
-      </c>
-      <c r="E12" s="6" t="s">
+      <c r="D12">
+        <v>13</v>
+      </c>
+      <c r="E12" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="4">
+      <c r="A13" s="2">
         <v>9299</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13">
         <v>4948</v>
       </c>
-      <c r="D13" s="6">
-        <v>13</v>
-      </c>
-      <c r="E13" s="6" t="s">
+      <c r="D13">
+        <v>13</v>
+      </c>
+      <c r="E13" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="4">
+      <c r="A14" s="2">
         <v>9073</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="6">
+      <c r="B14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14">
         <v>14902</v>
       </c>
-      <c r="D14" s="6">
-        <v>13</v>
-      </c>
-      <c r="E14" s="6" t="s">
+      <c r="D14">
+        <v>13</v>
+      </c>
+      <c r="E14" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="4">
+      <c r="A15" s="2">
         <v>9010</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15">
         <v>30780</v>
       </c>
-      <c r="D15" s="6">
-        <v>13</v>
-      </c>
-      <c r="E15" s="6" t="s">
+      <c r="D15">
+        <v>13</v>
+      </c>
+      <c r="E15" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="4">
+      <c r="A16" s="2">
         <v>9011</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16">
         <v>30913</v>
       </c>
-      <c r="D16" s="6">
-        <v>13</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B17" s="1"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D16">
+        <v>13</v>
+      </c>
+      <c r="E16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
+        <v>15721</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17">
+        <v>30780</v>
+      </c>
+      <c r="D17">
+        <v>13</v>
+      </c>
+      <c r="E17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B22" s="1"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B32" s="1"/>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>